<commit_message>
add filter feature project page
</commit_message>
<xml_diff>
--- a/public/BrandData/brand.xlsx
+++ b/public/BrandData/brand.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>ID</t>
   </si>
@@ -57,15 +57,6 @@
     <t>NIK</t>
   </si>
   <si>
-    <t>tina</t>
-  </si>
-  <si>
-    <t>tina@gmail.com</t>
-  </si>
-  <si>
-    <t>ksdkjnemekmcmklmwn</t>
-  </si>
-  <si>
     <t>098653244</t>
   </si>
   <si>
@@ -93,50 +84,26 @@
     <t>test</t>
   </si>
   <si>
-    <t>test1@gmail.com</t>
-  </si>
-  <si>
-    <t>jl. Tese</t>
-  </si>
-  <si>
-    <t>Beauty</t>
-  </si>
-  <si>
-    <t>123123</t>
-  </si>
-  <si>
-    <t>test bank</t>
-  </si>
-  <si>
-    <t>12.121.212.1-212.121</t>
-  </si>
-  <si>
-    <t>1212121212121212</t>
-  </si>
-  <si>
-    <t>test2</t>
-  </si>
-  <si>
-    <t>test2@gmail.com</t>
-  </si>
-  <si>
-    <t>jl. Test</t>
-  </si>
-  <si>
-    <t>test 2 bank</t>
-  </si>
-  <si>
-    <t>22.222.222.2-222.222</t>
+    <t>test@gmail.com</t>
+  </si>
+  <si>
+    <t>jakarta</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -157,14 +124,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -223,7 +192,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -258,7 +227,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -467,10 +436,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="24.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
@@ -522,116 +492,52 @@
         <v>21</v>
       </c>
       <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
+      <c r="F2" t="s">
         <v>13</v>
       </c>
-      <c r="D2" t="s">
+      <c r="G2" t="s">
         <v>14</v>
       </c>
-      <c r="E2" t="s">
+      <c r="H2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" t="s">
+      <c r="I2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" t="s">
+      <c r="J2" t="s">
         <v>17</v>
       </c>
-      <c r="H2" t="s">
+      <c r="K2" t="s">
         <v>18</v>
       </c>
-      <c r="I2" t="s">
+      <c r="L2" t="s">
         <v>19</v>
-      </c>
-      <c r="J2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>22</v>
-      </c>
-      <c r="B3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E3">
-        <v>12345678910</v>
-      </c>
-      <c r="F3" t="s">
-        <v>26</v>
-      </c>
-      <c r="G3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" t="s">
-        <v>27</v>
-      </c>
-      <c r="J3" t="s">
-        <v>28</v>
-      </c>
-      <c r="K3" t="s">
-        <v>29</v>
-      </c>
-      <c r="L3" t="s">
-        <v>30</v>
-      </c>
+      <c r="C3" s="1"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>23</v>
-      </c>
-      <c r="B4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D4" t="s">
-        <v>33</v>
-      </c>
-      <c r="E4">
-        <v>908923</v>
-      </c>
-      <c r="F4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H4" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4">
-        <v>189212918</v>
-      </c>
-      <c r="J4" t="s">
-        <v>34</v>
-      </c>
-      <c r="K4" t="s">
-        <v>35</v>
-      </c>
-      <c r="L4" s="1">
-        <v>1254512112121210</v>
-      </c>
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C5" s="1"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>